<commit_message>
Figures colonies & BS
</commit_message>
<xml_diff>
--- a/data/RawData/Effectif.xlsx
+++ b/data/RawData/Effectif.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ponchon\Documents\Projects\NorthernGannets2023\Analysis\NorthernGannets2023\data\RawData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BEFDDB3-2D71-475B-AC8D-60C308B109F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53DC80D0-0177-426B-B331-CB18451DC41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32310" yWindow="3510" windowWidth="21600" windowHeight="11385" xr2:uid="{A8D352B6-5B34-44B4-BCDC-16CF3AE2654A}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{A8D352B6-5B34-44B4-BCDC-16CF3AE2654A}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="2" r:id="rId1"/>
@@ -34,19 +34,22 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>year</t>
   </si>
   <si>
     <t>count</t>
   </si>
+  <si>
+    <t>success</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -62,6 +65,18 @@
     <font>
       <b/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color indexed="8"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -108,7 +123,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -134,6 +149,16 @@
     <xf numFmtId="3" fontId="2" fillId="2" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -449,98 +474,131 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72523CC1-0B69-4EC9-88B1-6876861858F6}">
-  <dimension ref="A1:B21"/>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>2023</v>
       </c>
       <c r="B2" s="7">
         <v>11592</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C2" s="9">
+        <v>0.5714285714285714</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>2022</v>
       </c>
       <c r="B3" s="5">
         <v>18747</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C3" s="10">
+        <v>2.9702970297029702E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2021</v>
       </c>
       <c r="B4" s="5">
         <v>18967</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C4" s="11">
+        <v>0.33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>2020</v>
       </c>
       <c r="B5" s="5">
         <v>21005</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C5" s="12">
+        <v>0.63207547169811318</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>2019</v>
       </c>
       <c r="B6" s="5">
         <v>21524</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C6" s="13">
+        <v>0.56310679611650483</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>2017</v>
       </c>
       <c r="B7" s="5">
         <v>18919</v>
       </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C7" s="14">
+        <v>0.32</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>2016</v>
       </c>
       <c r="B8" s="5">
         <v>20155</v>
       </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C8" s="15">
+        <v>0.42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>2015</v>
       </c>
       <c r="B9" s="8">
         <v>21217</v>
       </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C9" s="16">
+        <v>0.55000000000000004</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>2014</v>
       </c>
       <c r="B10" s="8">
         <v>21545</v>
       </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C10" s="17">
+        <v>0.62</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>2013</v>
       </c>
       <c r="B11" s="8">
         <v>19443</v>
       </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="C11" s="18">
+        <v>0.44</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>2012</v>
       </c>
@@ -548,7 +606,7 @@
         <v>20320</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>2011</v>
       </c>
@@ -556,7 +614,7 @@
         <v>22395</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>2010</v>
       </c>
@@ -564,7 +622,7 @@
         <v>21880</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>2009</v>
       </c>
@@ -572,7 +630,7 @@
         <v>21393</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>2008</v>
       </c>

</xml_diff>